<commit_message>
feat(F-NAR-016): TREE-DIF-038 passe agent après apply
</commit_message>
<xml_diff>
--- a/stories/arbres/TREE-DIF-038.xlsx
+++ b/stories/arbres/TREE-DIF-038.xlsx
@@ -2306,12 +2306,12 @@
       </c>
       <c r="E8" s="2" t="inlineStr">
         <is>
-          <t>Le cheval arrive près de l'établi. Le cheval bute contre un tas de copeaux. Des copeaux cachent les tiroirs, tout jaunes. C'est ici ? C'est le tiroir. Le mot s'arrête au milieu. Lequel ? Nino referme sa bouche, tout net. Les tiroirs se ressemblent tous. Vous faites comment, tous les deux ?</t>
+          <t>Le cheval arrive près de l'établi. Le cheval bute contre un tas de copeaux. Des copeaux cachent les tiroirs, tout jaunes. C'est ici ? C'est le tiroir. Le mot s'arrête au milieu. Lequel ? Nino referme sa bouche, tout net. Les tiroirs se ressemblent tous. On fait comment, Nino ?</t>
         </is>
       </c>
       <c r="F8" s="2" t="inlineStr">
         <is>
-          <t>Le cheval arrive près de l'établi. Le cheval bute contre un tas de copeaux. Des copeaux cachent les tiroirs, tout jaunes. C'est ici ? C'est le tiroir. Le mot s'arrête au milieu. Lequel ? Nino referme sa bouche, tout net. Les tiroirs se ressemblent tous. Vous faites comment, tous les deux ?</t>
+          <t>Le cheval arrive près de l'établi. Le cheval bute contre un tas de copeaux. Des copeaux cachent les tiroirs, tout jaunes. C'est ici ? C'est le tiroir. Le mot s'arrête au milieu. Lequel ? Nino referme sa bouche, tout net. Les tiroirs se ressemblent tous. On fait comment, Nino ?</t>
         </is>
       </c>
       <c r="G8" s="2" t="inlineStr">
@@ -2455,7 +2455,7 @@
 enfant-m|Lequel ?
 narrateur|Nino referme sa bouche, tout net.
 maman|Les tiroirs se ressemblent tous.
-papa|Vous faites comment, tous les deux ?</t>
+papa|On fait comment, Nino ?</t>
         </is>
       </c>
     </row>
@@ -3551,12 +3551,12 @@
       </c>
       <c r="E15" s="2" t="inlineStr">
         <is>
-          <t>La roue du bas tient, tout nette. On s'est baissés, papa. Le haut gardera son ombre. Lavez-vous les mains, tout doux. Le bois du cheval reste un peu tiède. Nino tapote le dos, tout léger. Le bois a un peu de poussière. Une abeille passe, puis l'auvent se tait.</t>
+          <t>La roue du bas tient, tout nette. On s'est baissés, papa. Le haut gardera son ombre. Lave-toi les mains, tout doux. Le bois du cheval reste un peu tiède. Nino tapote le dos, tout léger. Le bois a un peu de poussière. Une abeille passe, puis l'auvent se tait.</t>
         </is>
       </c>
       <c r="F15" s="2" t="inlineStr">
         <is>
-          <t>La roue du bas tient, tout nette. On s'est baissés, papa. Le haut gardera son ombre. Lavez-vous les mains, tout doux. Le bois du cheval reste un peu tiède. Nino tapote le dos, tout léger. Le bois a un peu de poussière. Une abeille passe, puis l'auvent se tait.</t>
+          <t>La roue du bas tient, tout nette. On s'est baissés, papa. Le haut gardera son ombre. Lave-toi les mains, tout doux. Le bois du cheval reste un peu tiède. Nino tapote le dos, tout léger. Le bois a un peu de poussière. Une abeille passe, puis l'auvent se tait.</t>
         </is>
       </c>
       <c r="G15" s="2" t="inlineStr">
@@ -3694,7 +3694,7 @@
           <t>narrateur|La roue du bas tient, tout nette.
 enfant-m|On s'est baissés, papa.
 papa|Le haut gardera son ombre.
-maman|Lavez-vous les mains, tout doux.
+maman|Lave-toi les mains, tout doux.
 narrateur|Le bois du cheval reste un peu tiède.
 narrateur|Nino tapote le dos, tout léger.
 narrateur|Le bois a un peu de poussière.
@@ -3725,12 +3725,12 @@
       </c>
       <c r="E16" s="2" t="inlineStr">
         <is>
-          <t>Le cheval arrive près du coffre. Le cheval penche contre le couvercle lourd. Elle est là-dedans ? Elle est dans le. Maman cherche, un doigt en l'air. Le couvercle ne bouge pas, encore. Ouvre ! Nino recule d'un pas, puis attend. Le bois est trop lourd, tout seul. Vous trouvez comment ?</t>
+          <t>Le cheval arrive près du coffre. Le cheval penche contre le couvercle lourd. Elle est là-dedans ? Elle est dans le. Maman cherche, un doigt en l'air. Le couvercle ne bouge pas, encore. Ouvre ! Nino recule d'un pas, puis attend. Le bois est trop lourd, tout seul. Tu trouves comment ?</t>
         </is>
       </c>
       <c r="F16" s="2" t="inlineStr">
         <is>
-          <t>Le cheval arrive près du coffre. Le cheval penche contre le couvercle lourd. Elle est là-dedans ? Elle est dans le. Maman cherche, un doigt en l'air. Le couvercle ne bouge pas, encore. Ouvre ! Nino recule d'un pas, puis attend. Le bois est trop lourd, tout seul. Vous trouvez comment ?</t>
+          <t>Le cheval arrive près du coffre. Le cheval penche contre le couvercle lourd. Elle est là-dedans ? Elle est dans le. Maman cherche, un doigt en l'air. Le couvercle ne bouge pas, encore. Ouvre ! Nino recule d'un pas, puis attend. Le bois est trop lourd, tout seul. Tu trouves comment ?</t>
         </is>
       </c>
       <c r="G16" s="2" t="inlineStr">
@@ -3874,7 +3874,7 @@
 enfant-m|Ouvre !
 narrateur|Nino recule d'un pas, puis attend.
 papa|Le bois est trop lourd, tout seul.
-maman|Vous trouvez comment ?</t>
+maman|Tu trouves comment ?</t>
         </is>
       </c>
     </row>
@@ -4445,12 +4445,12 @@
       </c>
       <c r="E20" s="2" t="inlineStr">
         <is>
-          <t>À deux. Tes mains ici, les miennes là. Le couvercle s'ouvre, tout lent. Dans le. Nino attend, les lèvres fermées. Dans le coin. Le cheval reste contre la jambe, tout sage. Vous avez porté ensemble. La suite a eu sa place.</t>
+          <t>À deux. Tes mains ici, les miennes là. Le couvercle s'ouvre, tout lent. Dans le. Nino attend, les lèvres fermées. Dans le coin. Le cheval reste contre la jambe, tout sage. On a porté ensemble. La suite a eu sa place.</t>
         </is>
       </c>
       <c r="F20" s="2" t="inlineStr">
         <is>
-          <t>À deux. Tes mains ici, les miennes là. Le couvercle s'ouvre, tout lent. Dans le. Nino attend, les lèvres fermées. Dans le coin. Le cheval reste contre la jambe, tout sage. Vous avez porté ensemble. La suite a eu sa place.</t>
+          <t>À deux. Tes mains ici, les miennes là. Le couvercle s'ouvre, tout lent. Dans le. Nino attend, les lèvres fermées. Dans le coin. Le cheval reste contre la jambe, tout sage. On a porté ensemble. La suite a eu sa place.</t>
         </is>
       </c>
       <c r="G20" s="2" t="inlineStr">
@@ -4592,7 +4592,7 @@
 narrateur|Nino attend, les lèvres fermées.
 maman|Dans le coin.
 narrateur|Le cheval reste contre la jambe, tout sage.
-papa|Vous avez porté ensemble.
+papa|On a porté ensemble.
 maman|La suite a eu sa place.</t>
         </is>
       </c>
@@ -4620,12 +4620,12 @@
       </c>
       <c r="E21" s="2" t="inlineStr">
         <is>
-          <t>À deux, le coffre a parlé, enfin. On a porté, tous les deux. Tes mains étaient à la bonne place. Le pain vous attend. Le bois du cheval reste un peu tiède. Nino essuie une main sur son pantalon. Un grain de savon reste sur le bois. Le cheval avance, roue après roue.</t>
+          <t>À deux, le coffre a parlé, enfin. On a porté, tous les deux. Tes mains étaient à la bonne place. Le pain t'attend. Le bois du cheval reste un peu tiède. Nino essuie une main sur son pantalon. Un grain de savon reste sur le bois. Le cheval avance, roue après roue.</t>
         </is>
       </c>
       <c r="F21" s="2" t="inlineStr">
         <is>
-          <t>À deux, le coffre a parlé, enfin. On a porté, tous les deux. Tes mains étaient à la bonne place. Le pain vous attend. Le bois du cheval reste un peu tiède. Nino essuie une main sur son pantalon. Un grain de savon reste sur le bois. Le cheval avance, roue après roue.</t>
+          <t>À deux, le coffre a parlé, enfin. On a porté, tous les deux. Tes mains étaient à la bonne place. Le pain t'attend. Le bois du cheval reste un peu tiède. Nino essuie une main sur son pantalon. Un grain de savon reste sur le bois. Le cheval avance, roue après roue.</t>
         </is>
       </c>
       <c r="G21" s="2" t="inlineStr">
@@ -4763,7 +4763,7 @@
           <t>narrateur|À deux, le coffre a parlé, enfin.
 enfant-m|On a porté, tous les deux.
 papa|Tes mains étaient à la bonne place.
-maman|Le pain vous attend.
+maman|Le pain t'attend.
 narrateur|Le bois du cheval reste un peu tiède.
 narrateur|Nino essuie une main sur son pantalon.
 narrateur|Un grain de savon reste sur le bois.
@@ -4794,12 +4794,12 @@
       </c>
       <c r="E22" s="2" t="inlineStr">
         <is>
-          <t>La cale, dessous. Je glisse le bois, tout doux. Le couvercle reste ouvert, un peu. À gauche. Nino tourne la tête, sans parler. Je la vois, au fond. Le cheval reste contre la jambe, tout sage. La cale a tenu le mot. Vous avez regardé ensemble.</t>
+          <t>La cale, dessous. Je glisse le bois, tout doux. Le couvercle reste ouvert, un peu. À gauche. Nino tourne la tête, sans parler. Je la vois, au fond. Le cheval reste contre la jambe, tout sage. La cale a tenu le mot. On a regardé ensemble.</t>
         </is>
       </c>
       <c r="F22" s="2" t="inlineStr">
         <is>
-          <t>La cale, dessous. Je glisse le bois, tout doux. Le couvercle reste ouvert, un peu. À gauche. Nino tourne la tête, sans parler. Je la vois, au fond. Le cheval reste contre la jambe, tout sage. La cale a tenu le mot. Vous avez regardé ensemble.</t>
+          <t>La cale, dessous. Je glisse le bois, tout doux. Le couvercle reste ouvert, un peu. À gauche. Nino tourne la tête, sans parler. Je la vois, au fond. Le cheval reste contre la jambe, tout sage. La cale a tenu le mot. On a regardé ensemble.</t>
         </is>
       </c>
       <c r="G22" s="2" t="inlineStr">
@@ -4942,7 +4942,7 @@
 enfant-m|Je la vois, au fond.
 narrateur|Le cheval reste contre la jambe, tout sage.
 papa|La cale a tenu le mot.
-maman|Vous avez regardé ensemble.</t>
+maman|On a regardé ensemble.</t>
         </is>
       </c>
     </row>
@@ -5143,12 +5143,12 @@
       </c>
       <c r="E24" s="2" t="inlineStr">
         <is>
-          <t>Le cheval arrive sous l'étagère. Le cheval lève le nez, trop bas encore. Tout en haut ? Tout en haut, près du. Papa s'arrête, les lèvres encore rondes. Près du pot ? Nino garde sa bouche fermée, après. Le haut est trop loin, pour lui. Un tabouret dort près du mur. Vous faites quoi, alors ?</t>
+          <t>Le cheval arrive sous l'étagère. Le cheval lève le nez, trop bas encore. Tout en haut ? Tout en haut, près du. Papa s'arrête, les lèvres encore rondes. Près du pot ? Nino garde sa bouche fermée, après. Le haut est trop loin, pour lui. Un tabouret dort près du mur. Tu fais quoi, alors ?</t>
         </is>
       </c>
       <c r="F24" s="2" t="inlineStr">
         <is>
-          <t>Le cheval arrive sous l'étagère. Le cheval lève le nez, trop bas encore. Tout en haut ? Tout en haut, près du. Papa s'arrête, les lèvres encore rondes. Près du pot ? Nino garde sa bouche fermée, après. Le haut est trop loin, pour lui. Un tabouret dort près du mur. Vous faites quoi, alors ?</t>
+          <t>Le cheval arrive sous l'étagère. Le cheval lève le nez, trop bas encore. Tout en haut ? Tout en haut, près du. Papa s'arrête, les lèvres encore rondes. Près du pot ? Nino garde sa bouche fermée, après. Le haut est trop loin, pour lui. Un tabouret dort près du mur. Tu fais quoi, alors ?</t>
         </is>
       </c>
       <c r="G24" s="2" t="inlineStr">
@@ -5292,7 +5292,7 @@
 narrateur|Nino garde sa bouche fermée, après.
 maman|Le haut est trop loin, pour lui.
 papa|Un tabouret dort près du mur.
-papa|Vous faites quoi, alors ?</t>
+papa|Tu fais quoi, alors ?</t>
         </is>
       </c>
     </row>
@@ -6927,12 +6927,12 @@
       </c>
       <c r="E34" s="2" t="inlineStr">
         <is>
-          <t>La boîte. Oui. Le cheval penche déjà sous le bras. Le chiffon dort dans la poche. Le métal a un peu sonné. J'écoute la suite. Vous restez ensemble.</t>
+          <t>La boîte. Oui. Le cheval penche déjà sous le bras. Le chiffon dort dans la poche. Le métal a un peu sonné. J'écoute la suite. On reste ensemble.</t>
         </is>
       </c>
       <c r="F34" s="2" t="inlineStr">
         <is>
-          <t>La boîte. Oui. Le cheval penche déjà sous le bras. Le chiffon dort dans la poche. Le métal a un peu sonné. J'écoute la suite. Vous restez ensemble.</t>
+          <t>La boîte. Oui. Le cheval penche déjà sous le bras. Le chiffon dort dans la poche. Le métal a un peu sonné. J'écoute la suite. On reste ensemble.</t>
         </is>
       </c>
       <c r="G34" s="2" t="inlineStr">
@@ -7077,7 +7077,7 @@
 narrateur|Le chiffon dort dans la poche.
 papa|Le métal a un peu sonné.
 enfant-m|J'écoute la suite.
-maman|Vous restez ensemble.</t>
+maman|On reste ensemble.</t>
         </is>
       </c>
     </row>
@@ -7297,12 +7297,12 @@
       </c>
       <c r="E36" s="2" t="inlineStr">
         <is>
-          <t>La boîte arrive près de l'établi. La boîte glisse sur une planche, tout fin. Des copeaux cachent les tiroirs, tout jaunes. C'est ici ? C'est le tiroir. Le mot s'arrête au milieu. Lequel ? Nino referme sa bouche, tout net. Les tiroirs se ressemblent tous. Vous faites comment, tous les deux ?</t>
+          <t>La boîte arrive près de l'établi. La boîte glisse sur une planche, tout fin. Des copeaux cachent les tiroirs, tout jaunes. C'est ici ? C'est le tiroir. Le mot s'arrête au milieu. Lequel ? Nino referme sa bouche, tout net. Les tiroirs se ressemblent tous. On fait comment, Nino ?</t>
         </is>
       </c>
       <c r="F36" s="2" t="inlineStr">
         <is>
-          <t>La boîte arrive près de l'établi. La boîte glisse sur une planche, tout fin. Des copeaux cachent les tiroirs, tout jaunes. C'est ici ? C'est le tiroir. Le mot s'arrête au milieu. Lequel ? Nino referme sa bouche, tout net. Les tiroirs se ressemblent tous. Vous faites comment, tous les deux ?</t>
+          <t>La boîte arrive près de l'établi. La boîte glisse sur une planche, tout fin. Des copeaux cachent les tiroirs, tout jaunes. C'est ici ? C'est le tiroir. Le mot s'arrête au milieu. Lequel ? Nino referme sa bouche, tout net. Les tiroirs se ressemblent tous. On fait comment, Nino ?</t>
         </is>
       </c>
       <c r="G36" s="2" t="inlineStr">
@@ -7446,7 +7446,7 @@
 enfant-m|Lequel ?
 narrateur|Nino referme sa bouche, tout net.
 maman|Les tiroirs se ressemblent tous.
-papa|Vous faites comment, tous les deux ?</t>
+papa|On fait comment, Nino ?</t>
         </is>
       </c>
     </row>
@@ -8542,12 +8542,12 @@
       </c>
       <c r="E43" s="2" t="inlineStr">
         <is>
-          <t>La roue du bas tient, tout nette. On s'est baissés, papa. Le haut gardera son ombre. Lavez-vous les mains, tout doux. La boîte ronde garde une poussière, tout fine. Nino tapote le dos, tout léger. Le bois a un peu de poussière. Une abeille passe, puis l'auvent se tait.</t>
+          <t>La roue du bas tient, tout nette. On s'est baissés, papa. Le haut gardera son ombre. Lave-toi les mains, tout doux. La boîte ronde garde une poussière, tout fine. Nino tapote le dos, tout léger. Le bois a un peu de poussière. Une abeille passe, puis l'auvent se tait.</t>
         </is>
       </c>
       <c r="F43" s="2" t="inlineStr">
         <is>
-          <t>La roue du bas tient, tout nette. On s'est baissés, papa. Le haut gardera son ombre. Lavez-vous les mains, tout doux. La boîte ronde garde une poussière, tout fine. Nino tapote le dos, tout léger. Le bois a un peu de poussière. Une abeille passe, puis l'auvent se tait.</t>
+          <t>La roue du bas tient, tout nette. On s'est baissés, papa. Le haut gardera son ombre. Lave-toi les mains, tout doux. La boîte ronde garde une poussière, tout fine. Nino tapote le dos, tout léger. Le bois a un peu de poussière. Une abeille passe, puis l'auvent se tait.</t>
         </is>
       </c>
       <c r="G43" s="2" t="inlineStr">
@@ -8685,7 +8685,7 @@
           <t>narrateur|La roue du bas tient, tout nette.
 enfant-m|On s'est baissés, papa.
 papa|Le haut gardera son ombre.
-maman|Lavez-vous les mains, tout doux.
+maman|Lave-toi les mains, tout doux.
 narrateur|La boîte ronde garde une poussière, tout fine.
 narrateur|Nino tapote le dos, tout léger.
 narrateur|Le bois a un peu de poussière.
@@ -8716,12 +8716,12 @@
       </c>
       <c r="E44" s="2" t="inlineStr">
         <is>
-          <t>La boîte arrive près du coffre. La boîte tape le bois, un petit toc. Elle est là-dedans ? Elle est dans le. Maman cherche, un doigt en l'air. Le couvercle ne bouge pas, encore. Ouvre ! Nino recule d'un pas, puis attend. Le bois est trop lourd, tout seul. Vous trouvez comment ?</t>
+          <t>La boîte arrive près du coffre. La boîte tape le bois, un petit toc. Elle est là-dedans ? Elle est dans le. Maman cherche, un doigt en l'air. Le couvercle ne bouge pas, encore. Ouvre ! Nino recule d'un pas, puis attend. Le bois est trop lourd, tout seul. Tu trouves comment ?</t>
         </is>
       </c>
       <c r="F44" s="2" t="inlineStr">
         <is>
-          <t>La boîte arrive près du coffre. La boîte tape le bois, un petit toc. Elle est là-dedans ? Elle est dans le. Maman cherche, un doigt en l'air. Le couvercle ne bouge pas, encore. Ouvre ! Nino recule d'un pas, puis attend. Le bois est trop lourd, tout seul. Vous trouvez comment ?</t>
+          <t>La boîte arrive près du coffre. La boîte tape le bois, un petit toc. Elle est là-dedans ? Elle est dans le. Maman cherche, un doigt en l'air. Le couvercle ne bouge pas, encore. Ouvre ! Nino recule d'un pas, puis attend. Le bois est trop lourd, tout seul. Tu trouves comment ?</t>
         </is>
       </c>
       <c r="G44" s="2" t="inlineStr">
@@ -8865,7 +8865,7 @@
 enfant-m|Ouvre !
 narrateur|Nino recule d'un pas, puis attend.
 papa|Le bois est trop lourd, tout seul.
-maman|Vous trouvez comment ?</t>
+maman|Tu trouves comment ?</t>
         </is>
       </c>
     </row>
@@ -9436,12 +9436,12 @@
       </c>
       <c r="E48" s="2" t="inlineStr">
         <is>
-          <t>À deux. Tes mains ici, les miennes là. Le couvercle s'ouvre, tout lent. Dans le. Nino attend, les lèvres fermées. Dans le coin. La boîte attend un dernier toc. Vous avez porté ensemble. La suite a eu sa place.</t>
+          <t>À deux. Tes mains ici, les miennes là. Le couvercle s'ouvre, tout lent. Dans le. Nino attend, les lèvres fermées. Dans le coin. La boîte attend un dernier toc. On a porté ensemble. La suite a eu sa place.</t>
         </is>
       </c>
       <c r="F48" s="2" t="inlineStr">
         <is>
-          <t>À deux. Tes mains ici, les miennes là. Le couvercle s'ouvre, tout lent. Dans le. Nino attend, les lèvres fermées. Dans le coin. La boîte attend un dernier toc. Vous avez porté ensemble. La suite a eu sa place.</t>
+          <t>À deux. Tes mains ici, les miennes là. Le couvercle s'ouvre, tout lent. Dans le. Nino attend, les lèvres fermées. Dans le coin. La boîte attend un dernier toc. On a porté ensemble. La suite a eu sa place.</t>
         </is>
       </c>
       <c r="G48" s="2" t="inlineStr">
@@ -9583,7 +9583,7 @@
 narrateur|Nino attend, les lèvres fermées.
 maman|Dans le coin.
 narrateur|La boîte attend un dernier toc.
-papa|Vous avez porté ensemble.
+papa|On a porté ensemble.
 maman|La suite a eu sa place.</t>
         </is>
       </c>
@@ -9611,12 +9611,12 @@
       </c>
       <c r="E49" s="2" t="inlineStr">
         <is>
-          <t>À deux, le coffre a parlé, enfin. On a porté, tous les deux. Tes mains étaient à la bonne place. Le pain vous attend. La boîte ronde garde une poussière, tout fine. Nino essuie une main sur son pantalon. Un grain de savon reste sur le bois. Le cheval avance, roue après roue.</t>
+          <t>À deux, le coffre a parlé, enfin. On a porté, tous les deux. Tes mains étaient à la bonne place. Le pain t'attend. La boîte ronde garde une poussière, tout fine. Nino essuie une main sur son pantalon. Un grain de savon reste sur le bois. Le cheval avance, roue après roue.</t>
         </is>
       </c>
       <c r="F49" s="2" t="inlineStr">
         <is>
-          <t>À deux, le coffre a parlé, enfin. On a porté, tous les deux. Tes mains étaient à la bonne place. Le pain vous attend. La boîte ronde garde une poussière, tout fine. Nino essuie une main sur son pantalon. Un grain de savon reste sur le bois. Le cheval avance, roue après roue.</t>
+          <t>À deux, le coffre a parlé, enfin. On a porté, tous les deux. Tes mains étaient à la bonne place. Le pain t'attend. La boîte ronde garde une poussière, tout fine. Nino essuie une main sur son pantalon. Un grain de savon reste sur le bois. Le cheval avance, roue après roue.</t>
         </is>
       </c>
       <c r="G49" s="2" t="inlineStr">
@@ -9754,7 +9754,7 @@
           <t>narrateur|À deux, le coffre a parlé, enfin.
 enfant-m|On a porté, tous les deux.
 papa|Tes mains étaient à la bonne place.
-maman|Le pain vous attend.
+maman|Le pain t'attend.
 narrateur|La boîte ronde garde une poussière, tout fine.
 narrateur|Nino essuie une main sur son pantalon.
 narrateur|Un grain de savon reste sur le bois.
@@ -9785,12 +9785,12 @@
       </c>
       <c r="E50" s="2" t="inlineStr">
         <is>
-          <t>La cale, dessous. Je glisse le bois, tout doux. Le couvercle reste ouvert, un peu. À gauche. Nino tourne la tête, sans parler. Je la vois, au fond. La boîte attend un dernier toc. La cale a tenu le mot. Vous avez regardé ensemble.</t>
+          <t>La cale, dessous. Je glisse le bois, tout doux. Le couvercle reste ouvert, un peu. À gauche. Nino tourne la tête, sans parler. Je la vois, au fond. La boîte attend un dernier toc. La cale a tenu le mot. On a regardé ensemble.</t>
         </is>
       </c>
       <c r="F50" s="2" t="inlineStr">
         <is>
-          <t>La cale, dessous. Je glisse le bois, tout doux. Le couvercle reste ouvert, un peu. À gauche. Nino tourne la tête, sans parler. Je la vois, au fond. La boîte attend un dernier toc. La cale a tenu le mot. Vous avez regardé ensemble.</t>
+          <t>La cale, dessous. Je glisse le bois, tout doux. Le couvercle reste ouvert, un peu. À gauche. Nino tourne la tête, sans parler. Je la vois, au fond. La boîte attend un dernier toc. La cale a tenu le mot. On a regardé ensemble.</t>
         </is>
       </c>
       <c r="G50" s="2" t="inlineStr">
@@ -9933,7 +9933,7 @@
 enfant-m|Je la vois, au fond.
 narrateur|La boîte attend un dernier toc.
 papa|La cale a tenu le mot.
-maman|Vous avez regardé ensemble.</t>
+maman|On a regardé ensemble.</t>
         </is>
       </c>
     </row>
@@ -10134,12 +10134,12 @@
       </c>
       <c r="E52" s="2" t="inlineStr">
         <is>
-          <t>La boîte arrive sous l'étagère. La boîte n'atteint pas le bord, trop haute. Tout en haut ? Tout en haut, près du. Papa s'arrête, les lèvres encore rondes. Près du pot ? Nino garde sa bouche fermée, après. Le haut est trop loin, pour lui. Un tabouret dort près du mur. Vous faites quoi, alors ?</t>
+          <t>La boîte arrive sous l'étagère. La boîte n'atteint pas le bord, trop haute. Tout en haut ? Tout en haut, près du. Papa s'arrête, les lèvres encore rondes. Près du pot ? Nino garde sa bouche fermée, après. Le haut est trop loin, pour lui. Un tabouret dort près du mur. Tu fais quoi, alors ?</t>
         </is>
       </c>
       <c r="F52" s="2" t="inlineStr">
         <is>
-          <t>La boîte arrive sous l'étagère. La boîte n'atteint pas le bord, trop haute. Tout en haut ? Tout en haut, près du. Papa s'arrête, les lèvres encore rondes. Près du pot ? Nino garde sa bouche fermée, après. Le haut est trop loin, pour lui. Un tabouret dort près du mur. Vous faites quoi, alors ?</t>
+          <t>La boîte arrive sous l'étagère. La boîte n'atteint pas le bord, trop haute. Tout en haut ? Tout en haut, près du. Papa s'arrête, les lèvres encore rondes. Près du pot ? Nino garde sa bouche fermée, après. Le haut est trop loin, pour lui. Un tabouret dort près du mur. Tu fais quoi, alors ?</t>
         </is>
       </c>
       <c r="G52" s="2" t="inlineStr">
@@ -10283,7 +10283,7 @@
 narrateur|Nino garde sa bouche fermée, après.
 maman|Le haut est trop loin, pour lui.
 papa|Un tabouret dort près du mur.
-papa|Vous faites quoi, alors ?</t>
+papa|Tu fais quoi, alors ?</t>
         </is>
       </c>
     </row>
@@ -12288,12 +12288,12 @@
       </c>
       <c r="E64" s="2" t="inlineStr">
         <is>
-          <t>Le chiffon arrive près de l'établi. Le chiffon s'accroche à une écharde. Des copeaux cachent les tiroirs, tout jaunes. C'est ici ? C'est le tiroir. Le mot s'arrête au milieu. Lequel ? Nino referme sa bouche, tout net. Les tiroirs se ressemblent tous. Vous faites comment, tous les deux ?</t>
+          <t>Le chiffon arrive près de l'établi. Le chiffon s'accroche à une écharde. Des copeaux cachent les tiroirs, tout jaunes. C'est ici ? C'est le tiroir. Le mot s'arrête au milieu. Lequel ? Nino referme sa bouche, tout net. Les tiroirs se ressemblent tous. On fait comment, Nino ?</t>
         </is>
       </c>
       <c r="F64" s="2" t="inlineStr">
         <is>
-          <t>Le chiffon arrive près de l'établi. Le chiffon s'accroche à une écharde. Des copeaux cachent les tiroirs, tout jaunes. C'est ici ? C'est le tiroir. Le mot s'arrête au milieu. Lequel ? Nino referme sa bouche, tout net. Les tiroirs se ressemblent tous. Vous faites comment, tous les deux ?</t>
+          <t>Le chiffon arrive près de l'établi. Le chiffon s'accroche à une écharde. Des copeaux cachent les tiroirs, tout jaunes. C'est ici ? C'est le tiroir. Le mot s'arrête au milieu. Lequel ? Nino referme sa bouche, tout net. Les tiroirs se ressemblent tous. On fait comment, Nino ?</t>
         </is>
       </c>
       <c r="G64" s="2" t="inlineStr">
@@ -12437,7 +12437,7 @@
 enfant-m|Lequel ?
 narrateur|Nino referme sa bouche, tout net.
 maman|Les tiroirs se ressemblent tous.
-papa|Vous faites comment, tous les deux ?</t>
+papa|On fait comment, Nino ?</t>
         </is>
       </c>
     </row>
@@ -13533,12 +13533,12 @@
       </c>
       <c r="E71" s="2" t="inlineStr">
         <is>
-          <t>La roue du bas tient, tout nette. On s'est baissés, papa. Le haut gardera son ombre. Lavez-vous les mains, tout doux. Le chiffon sent encore le savon du bois. Nino tapote le dos, tout léger. Le bois a un peu de poussière. Une abeille passe, puis l'auvent se tait.</t>
+          <t>La roue du bas tient, tout nette. On s'est baissés, papa. Le haut gardera son ombre. Lave-toi les mains, tout doux. Le chiffon sent encore le savon du bois. Nino tapote le dos, tout léger. Le bois a un peu de poussière. Une abeille passe, puis l'auvent se tait.</t>
         </is>
       </c>
       <c r="F71" s="2" t="inlineStr">
         <is>
-          <t>La roue du bas tient, tout nette. On s'est baissés, papa. Le haut gardera son ombre. Lavez-vous les mains, tout doux. Le chiffon sent encore le savon du bois. Nino tapote le dos, tout léger. Le bois a un peu de poussière. Une abeille passe, puis l'auvent se tait.</t>
+          <t>La roue du bas tient, tout nette. On s'est baissés, papa. Le haut gardera son ombre. Lave-toi les mains, tout doux. Le chiffon sent encore le savon du bois. Nino tapote le dos, tout léger. Le bois a un peu de poussière. Une abeille passe, puis l'auvent se tait.</t>
         </is>
       </c>
       <c r="G71" s="2" t="inlineStr">
@@ -13676,7 +13676,7 @@
           <t>narrateur|La roue du bas tient, tout nette.
 enfant-m|On s'est baissés, papa.
 papa|Le haut gardera son ombre.
-maman|Lavez-vous les mains, tout doux.
+maman|Lave-toi les mains, tout doux.
 narrateur|Le chiffon sent encore le savon du bois.
 narrateur|Nino tapote le dos, tout léger.
 narrateur|Le bois a un peu de poussière.
@@ -13707,12 +13707,12 @@
       </c>
       <c r="E72" s="2" t="inlineStr">
         <is>
-          <t>Le chiffon arrive près du coffre. Le chiffon glisse sous le bord, déjà. Elle est là-dedans ? Elle est dans le. Maman cherche, un doigt en l'air. Le couvercle ne bouge pas, encore. Ouvre ! Nino recule d'un pas, puis attend. Le bois est trop lourd, tout seul. Vous trouvez comment ?</t>
+          <t>Le chiffon arrive près du coffre. Le chiffon glisse sous le bord, déjà. Elle est là-dedans ? Elle est dans le. Maman cherche, un doigt en l'air. Le couvercle ne bouge pas, encore. Ouvre ! Nino recule d'un pas, puis attend. Le bois est trop lourd, tout seul. Tu trouves comment ?</t>
         </is>
       </c>
       <c r="F72" s="2" t="inlineStr">
         <is>
-          <t>Le chiffon arrive près du coffre. Le chiffon glisse sous le bord, déjà. Elle est là-dedans ? Elle est dans le. Maman cherche, un doigt en l'air. Le couvercle ne bouge pas, encore. Ouvre ! Nino recule d'un pas, puis attend. Le bois est trop lourd, tout seul. Vous trouvez comment ?</t>
+          <t>Le chiffon arrive près du coffre. Le chiffon glisse sous le bord, déjà. Elle est là-dedans ? Elle est dans le. Maman cherche, un doigt en l'air. Le couvercle ne bouge pas, encore. Ouvre ! Nino recule d'un pas, puis attend. Le bois est trop lourd, tout seul. Tu trouves comment ?</t>
         </is>
       </c>
       <c r="G72" s="2" t="inlineStr">
@@ -13856,7 +13856,7 @@
 enfant-m|Ouvre !
 narrateur|Nino recule d'un pas, puis attend.
 papa|Le bois est trop lourd, tout seul.
-maman|Vous trouvez comment ?</t>
+maman|Tu trouves comment ?</t>
         </is>
       </c>
     </row>
@@ -14427,12 +14427,12 @@
       </c>
       <c r="E76" s="2" t="inlineStr">
         <is>
-          <t>À deux. Tes mains ici, les miennes là. Le couvercle s'ouvre, tout lent. Dans le. Nino attend, les lèvres fermées. Dans le coin. Le chiffon dort contre sa paume. Vous avez porté ensemble. La suite a eu sa place.</t>
+          <t>À deux. Tes mains ici, les miennes là. Le couvercle s'ouvre, tout lent. Dans le. Nino attend, les lèvres fermées. Dans le coin. Le chiffon dort contre sa paume. On a porté ensemble. La suite a eu sa place.</t>
         </is>
       </c>
       <c r="F76" s="2" t="inlineStr">
         <is>
-          <t>À deux. Tes mains ici, les miennes là. Le couvercle s'ouvre, tout lent. Dans le. Nino attend, les lèvres fermées. Dans le coin. Le chiffon dort contre sa paume. Vous avez porté ensemble. La suite a eu sa place.</t>
+          <t>À deux. Tes mains ici, les miennes là. Le couvercle s'ouvre, tout lent. Dans le. Nino attend, les lèvres fermées. Dans le coin. Le chiffon dort contre sa paume. On a porté ensemble. La suite a eu sa place.</t>
         </is>
       </c>
       <c r="G76" s="2" t="inlineStr">
@@ -14574,7 +14574,7 @@
 narrateur|Nino attend, les lèvres fermées.
 maman|Dans le coin.
 narrateur|Le chiffon dort contre sa paume.
-papa|Vous avez porté ensemble.
+papa|On a porté ensemble.
 maman|La suite a eu sa place.</t>
         </is>
       </c>
@@ -14602,12 +14602,12 @@
       </c>
       <c r="E77" s="2" t="inlineStr">
         <is>
-          <t>À deux, le coffre a parlé, enfin. On a porté, tous les deux. Tes mains étaient à la bonne place. Le pain vous attend. Le chiffon sent encore le savon du bois. Nino essuie une main sur son pantalon. Un grain de savon reste sur le bois. Le cheval avance, roue après roue.</t>
+          <t>À deux, le coffre a parlé, enfin. On a porté, tous les deux. Tes mains étaient à la bonne place. Le pain t'attend. Le chiffon sent encore le savon du bois. Nino essuie une main sur son pantalon. Un grain de savon reste sur le bois. Le cheval avance, roue après roue.</t>
         </is>
       </c>
       <c r="F77" s="2" t="inlineStr">
         <is>
-          <t>À deux, le coffre a parlé, enfin. On a porté, tous les deux. Tes mains étaient à la bonne place. Le pain vous attend. Le chiffon sent encore le savon du bois. Nino essuie une main sur son pantalon. Un grain de savon reste sur le bois. Le cheval avance, roue après roue.</t>
+          <t>À deux, le coffre a parlé, enfin. On a porté, tous les deux. Tes mains étaient à la bonne place. Le pain t'attend. Le chiffon sent encore le savon du bois. Nino essuie une main sur son pantalon. Un grain de savon reste sur le bois. Le cheval avance, roue après roue.</t>
         </is>
       </c>
       <c r="G77" s="2" t="inlineStr">
@@ -14745,7 +14745,7 @@
           <t>narrateur|À deux, le coffre a parlé, enfin.
 enfant-m|On a porté, tous les deux.
 papa|Tes mains étaient à la bonne place.
-maman|Le pain vous attend.
+maman|Le pain t'attend.
 narrateur|Le chiffon sent encore le savon du bois.
 narrateur|Nino essuie une main sur son pantalon.
 narrateur|Un grain de savon reste sur le bois.
@@ -14776,12 +14776,12 @@
       </c>
       <c r="E78" s="2" t="inlineStr">
         <is>
-          <t>La cale, dessous. Je glisse le bois, tout doux. Le couvercle reste ouvert, un peu. À gauche. Nino tourne la tête, sans parler. Je la vois, au fond. Le chiffon dort contre sa paume. La cale a tenu le mot. Vous avez regardé ensemble.</t>
+          <t>La cale, dessous. Je glisse le bois, tout doux. Le couvercle reste ouvert, un peu. À gauche. Nino tourne la tête, sans parler. Je la vois, au fond. Le chiffon dort contre sa paume. La cale a tenu le mot. On a regardé ensemble.</t>
         </is>
       </c>
       <c r="F78" s="2" t="inlineStr">
         <is>
-          <t>La cale, dessous. Je glisse le bois, tout doux. Le couvercle reste ouvert, un peu. À gauche. Nino tourne la tête, sans parler. Je la vois, au fond. Le chiffon dort contre sa paume. La cale a tenu le mot. Vous avez regardé ensemble.</t>
+          <t>La cale, dessous. Je glisse le bois, tout doux. Le couvercle reste ouvert, un peu. À gauche. Nino tourne la tête, sans parler. Je la vois, au fond. Le chiffon dort contre sa paume. La cale a tenu le mot. On a regardé ensemble.</t>
         </is>
       </c>
       <c r="G78" s="2" t="inlineStr">
@@ -14924,7 +14924,7 @@
 enfant-m|Je la vois, au fond.
 narrateur|Le chiffon dort contre sa paume.
 papa|La cale a tenu le mot.
-maman|Vous avez regardé ensemble.</t>
+maman|On a regardé ensemble.</t>
         </is>
       </c>
     </row>
@@ -15125,12 +15125,12 @@
       </c>
       <c r="E80" s="2" t="inlineStr">
         <is>
-          <t>Le chiffon arrive sous l'étagère. Le chiffon pend, trop court, sous le bois. Tout en haut ? Tout en haut, près du. Papa s'arrête, les lèvres encore rondes. Près du pot ? Nino garde sa bouche fermée, après. Le haut est trop loin, pour lui. Un tabouret dort près du mur. Vous faites quoi, alors ?</t>
+          <t>Le chiffon arrive sous l'étagère. Le chiffon pend, trop court, sous le bois. Tout en haut ? Tout en haut, près du. Papa s'arrête, les lèvres encore rondes. Près du pot ? Nino garde sa bouche fermée, après. Le haut est trop loin, pour lui. Un tabouret dort près du mur. Tu fais quoi, alors ?</t>
         </is>
       </c>
       <c r="F80" s="2" t="inlineStr">
         <is>
-          <t>Le chiffon arrive sous l'étagère. Le chiffon pend, trop court, sous le bois. Tout en haut ? Tout en haut, près du. Papa s'arrête, les lèvres encore rondes. Près du pot ? Nino garde sa bouche fermée, après. Le haut est trop loin, pour lui. Un tabouret dort près du mur. Vous faites quoi, alors ?</t>
+          <t>Le chiffon arrive sous l'étagère. Le chiffon pend, trop court, sous le bois. Tout en haut ? Tout en haut, près du. Papa s'arrête, les lèvres encore rondes. Près du pot ? Nino garde sa bouche fermée, après. Le haut est trop loin, pour lui. Un tabouret dort près du mur. Tu fais quoi, alors ?</t>
         </is>
       </c>
       <c r="G80" s="2" t="inlineStr">
@@ -15274,7 +15274,7 @@
 narrateur|Nino garde sa bouche fermée, après.
 maman|Le haut est trop loin, pour lui.
 papa|Un tabouret dort près du mur.
-papa|Vous faites quoi, alors ?</t>
+papa|Tu fais quoi, alors ?</t>
         </is>
       </c>
     </row>
@@ -16537,7 +16537,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A14"/>
+  <dimension ref="A1:A15"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="100" customWidth="1" min="1" max="1"/>
@@ -16636,6 +16636,13 @@
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
+        <is>
+          <t>F-NAR-008 récit, pas une leçon en puces</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
         <is>
           <t>F-NAR-008 récit, pas une leçon en puces</t>
         </is>

</xml_diff>